<commit_message>
fix and add tailwind
</commit_message>
<xml_diff>
--- a/assets/savings-dashboard-demo.xlsx
+++ b/assets/savings-dashboard-demo.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="77">
   <si>
     <t>Savings Dashboard Demo / קובץ דוגמה למרכז החסכונות</t>
   </si>
@@ -98,7 +98,7 @@
     <t>O15:P20 store the historical totals used by the growth chart.</t>
   </si>
   <si>
-    <t>אחוז עליה</t>
+    <t>אחוז עליה נטו</t>
   </si>
   <si>
     <t>קופת גמל להשקעה</t>
@@ -125,6 +125,9 @@
     <t>מור</t>
   </si>
   <si>
+    <t>כולל הפקדות</t>
+  </si>
+  <si>
     <t>חיסכון לכל ילד</t>
   </si>
   <si>
@@ -132,6 +135,9 @@
   </si>
   <si>
     <t>דניאל</t>
+  </si>
+  <si>
+    <t>אחוז עליה הפקדות</t>
   </si>
   <si>
     <t>מסלול הלכה</t>
@@ -913,7 +919,7 @@
         <v>35500</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>34</v>
       </c>
@@ -932,13 +938,20 @@
       <c r="F10" s="7">
         <v>1800</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="O10" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="P10" s="7">
+        <f>SUM(F5:F16)</f>
+        <v>45200</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C11" s="7">
         <v>28400</v>
@@ -947,18 +960,25 @@
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F11" s="7">
         <v>900</v>
       </c>
+      <c r="O11" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="P11" s="10">
+        <f>IFERROR(P10/P7,0)</f>
+        <v>0.0428842504743833</v>
+      </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C12" s="7">
         <v>27100</v>
@@ -967,7 +987,7 @@
         <v>17</v>
       </c>
       <c r="E12" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F12" s="7">
         <v>900</v>
@@ -975,16 +995,16 @@
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B13" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C13" s="7">
         <v>123000</v>
       </c>
       <c r="D13" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E13" t="s">
         <v>13</v>
@@ -993,22 +1013,22 @@
         <v>5000</v>
       </c>
       <c r="O13" s="11" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="P13" s="11"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C14" s="7">
         <v>88000</v>
       </c>
       <c r="D14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E14" t="s">
         <v>32</v>
@@ -1017,7 +1037,7 @@
         <v>2500</v>
       </c>
       <c r="O14" s="11" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="P14" s="11" t="s">
         <v>4</v>
@@ -1025,16 +1045,16 @@
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B15" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C15" s="7">
         <v>45000</v>
       </c>
       <c r="D15" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E15" t="s">
         <v>32</v>
@@ -1043,7 +1063,7 @@
         <v>10000</v>
       </c>
       <c r="O15" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="P15" s="7">
         <v>910000</v>
@@ -1054,13 +1074,13 @@
         <v>29</v>
       </c>
       <c r="B16" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C16" s="7">
         <v>81000</v>
       </c>
       <c r="D16" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E16" t="s">
         <v>18</v>
@@ -1069,7 +1089,7 @@
         <v>2700</v>
       </c>
       <c r="O16" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="P16" s="7">
         <v>934500</v>
@@ -1077,7 +1097,7 @@
     </row>
     <row r="17" spans="15:16" x14ac:dyDescent="0.25">
       <c r="O17" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="P17" s="7">
         <v>962000</v>
@@ -1085,7 +1105,7 @@
     </row>
     <row r="18" spans="15:16" x14ac:dyDescent="0.25">
       <c r="O18" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="P18" s="7">
         <v>1001500</v>
@@ -1093,7 +1113,7 @@
     </row>
     <row r="19" spans="15:16" x14ac:dyDescent="0.25">
       <c r="O19" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="P19" s="7">
         <v>1054000</v>
@@ -1101,7 +1121,7 @@
     </row>
     <row r="20" spans="15:16" x14ac:dyDescent="0.25">
       <c r="O20" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="P20" s="7">
         <v>1089500</v>
@@ -1133,7 +1153,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B1" s="12"/>
       <c r="C1" s="12"/>
@@ -1145,7 +1165,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1157,13 +1177,13 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
@@ -1172,14 +1192,14 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B5" s="7">
         <f>sheet1!P5</f>
         <v>1089500</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E5" s="8"/>
       <c r="F5" s="8"/>
@@ -1188,14 +1208,14 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B6" s="7">
         <f>sheet1!P7</f>
         <v>1054000</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E6" s="9"/>
       <c r="F6" s="9"/>
@@ -1204,14 +1224,14 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B7" s="7">
         <f>sheet1!P9</f>
         <v>35500</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E7" s="8"/>
       <c r="F7" s="8"/>
@@ -1220,14 +1240,14 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B8" s="10">
         <f>sheet1!P8</f>
         <v>0.03368121442125238</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E8" s="9"/>
       <c r="F8" s="9"/>
@@ -1236,15 +1256,15 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B11" s="7">
         <v>910000</v>
@@ -1252,7 +1272,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B12" s="7">
         <v>934500</v>
@@ -1260,7 +1280,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B13" s="7">
         <v>962000</v>
@@ -1268,7 +1288,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B14" s="7">
         <v>1001500</v>
@@ -1276,7 +1296,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B15" s="7">
         <v>1054000</v>
@@ -1284,7 +1304,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B16" s="7">
         <v>1089500</v>

</xml_diff>